<commit_message>
update database with positive angles
</commit_message>
<xml_diff>
--- a/+results/Team Design Challenge 2026 (MSc Aerospace).xlsx
+++ b/+results/Team Design Challenge 2026 (MSc Aerospace).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\i2sc_LapTimeSimulator\+results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB0E57B-4C56-4D58-A12D-B260BF7FF9B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1E3775-6916-4A2E-8344-E6A6AA5341CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3380" yWindow="2740" windowWidth="21810" windowHeight="15380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -269,10 +269,10 @@
     <t>Dr Healy</t>
   </si>
   <si>
-    <t>2506</t>
-  </si>
-  <si>
-    <t>8315</t>
+    <t>2604</t>
+  </si>
+  <si>
+    <t>9313</t>
   </si>
 </sst>
 </file>
@@ -308,19 +308,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -332,12 +337,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -420,42 +419,42 @@
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Team Members" dataDxfId="2">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Team Members" dataDxfId="5">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r131430f88c284f6a86deab838a74d925"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Front Wing Airfoil Section" dataDxfId="0">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Front Wing Airfoil Section" dataDxfId="4">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rc1c9baf17b174995bc73c65461e272d3"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Front Wing Angle of Attack (deg)" dataDxfId="1">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Front Wing Angle of Attack (deg)" dataDxfId="3">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r5e90d4659e5f4ad694c35baa60518eb9"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Rear Wing Airfoil Section" dataDxfId="3">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Rear Wing Airfoil Section" dataDxfId="2">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rd7448ff9d5814691bfdc09b7ba11ab6a"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Rear Wing Angle of Attack (deg)" dataDxfId="4">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Rear Wing Angle of Attack (deg)" dataDxfId="1">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rf404bef8fe4542cc9d1a2e9fe19cc07d"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Gear Ratio Scaling " dataDxfId="5">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Gear Ratio Scaling " dataDxfId="0">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r0a81bd9db5b04c5d8d78495bb55f4a2a"/>
@@ -1159,28 +1158,27 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="5"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6" t="s">
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6" t="s">
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5" t="s">
         <v>77</v>
       </c>
       <c r="J10" s="2">
-        <v>-0.14099999999999999</v>
-      </c>
-      <c r="K10" s="6" t="s">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>78</v>
       </c>
       <c r="L10" s="2">
-        <v>-16.155999999999999</v>
+        <v>-14.875999999999999</v>
       </c>
       <c r="M10" s="2">
-        <v>1.0064</v>
+        <v>1.0072000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>